<commit_message>
Added sql model for measure inputs and pivoted load shapes and avoided cost models
</commit_message>
<xml_diff>
--- a/nspm/Input/OpenBCA Code PROGRAM INPUT.xlsx
+++ b/nspm/Input/OpenBCA Code PROGRAM INPUT.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://icfonlineapc-my.sharepoint.com/personal/59212_icf_com/Documents/Python Projects/OpenBCA_test_CK/nspm/Input/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://icfonlineapc-my.sharepoint.com/personal/59212_icf_com/Documents/Python Projects/openbca-2/nspm/Input/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="103383" documentId="11_4DDC0F817FA9BDDBAC50F43ADA4DC14C069E7AC6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DBE531E9-1C49-45CB-93A9-606C5F640E95}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="1330" yWindow="2930" windowWidth="14400" windowHeight="8170" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Front Page" sheetId="2" r:id="rId1"/>
@@ -9403,26 +9403,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="4724944d-d052-4dc6-ba96-b334b2cd88d4">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="fba8dc25-c80a-45e7-8728-03162ad94bfc" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100303C18EB8DAB7840BDA4B7C087A71E86" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="c385ee6626827eff31a893e8549e105a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="4724944d-d052-4dc6-ba96-b334b2cd88d4" xmlns:ns3="fba8dc25-c80a-45e7-8728-03162ad94bfc" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="efc1c5a003d74c25c5063cd6cc92a936" ns2:_="" ns3:_="">
     <xsd:import namespace="4724944d-d052-4dc6-ba96-b334b2cd88d4"/>
@@ -9617,26 +9597,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D56C6BAF-97BF-40E3-A1CB-E8E1559A76B0}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="4724944d-d052-4dc6-ba96-b334b2cd88d4"/>
-    <ds:schemaRef ds:uri="fba8dc25-c80a-45e7-8728-03162ad94bfc"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2C0B5564-36C4-46D7-8383-8131ECCB1949}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="4724944d-d052-4dc6-ba96-b334b2cd88d4">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="fba8dc25-c80a-45e7-8728-03162ad94bfc" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{69A4A6DB-5C3E-45FC-B18D-98CED6CB396A}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -9653,4 +9634,23 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2C0B5564-36C4-46D7-8383-8131ECCB1949}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D56C6BAF-97BF-40E3-A1CB-E8E1559A76B0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="4724944d-d052-4dc6-ba96-b334b2cd88d4"/>
+    <ds:schemaRef ds:uri="fba8dc25-c80a-45e7-8728-03162ad94bfc"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>